<commit_message>
RPT MOTOR RUN-OK: LISTA JERARQUICA AREAS REPORTE 1.35
</commit_message>
<xml_diff>
--- a/docs/3.1.- planificacion_menus_crud_asistencia.xlsx
+++ b/docs/3.1.- planificacion_menus_crud_asistencia.xlsx
@@ -4,21 +4,24 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="735" yWindow="6075" windowWidth="4185" windowHeight="2130" activeTab="1"/>
+    <workbookView xWindow="735" yWindow="6075" windowWidth="4185" windowHeight="2130"/>
   </bookViews>
   <sheets>
-    <sheet name="Crono al 2026.08.16" sheetId="1" r:id="rId1"/>
-    <sheet name="reglas y params asistencia 1.02" sheetId="3" r:id="rId2"/>
+    <sheet name="Crono al 2026.09.02" sheetId="5" r:id="rId1"/>
+    <sheet name="Crono al 2026.08.16" sheetId="1" r:id="rId2"/>
+    <sheet name="reglas y params asistencia 1.03" sheetId="4" r:id="rId3"/>
+    <sheet name="reglas y params asistencia 1.02" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Crono al 2026.08.16'!$A$1:$N$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Crono al 2026.08.16'!$A$1:$N$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Crono al 2026.09.02'!$A$1:$O$44</definedName>
   </definedNames>
   <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="465">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1578" uniqueCount="475">
   <si>
     <t>Menú</t>
   </si>
@@ -1413,6 +1416,72 @@
   </si>
   <si>
     <t>nombre de horario, si empieza con HR=descuenta 60 min de refrigerio, HN=descuenta 90 min de refrigerio, HS o Cualquier otro prefijo=NO DESCUENTA REFRIGERIO DE FORMA AUTOMATICA</t>
+  </si>
+  <si>
+    <t>NO USADO</t>
+  </si>
+  <si>
+    <t>Permite activar Fin de Semana para procesar y mostrar H.E.</t>
+  </si>
+  <si>
+    <t>Permite programar que dias son Fin de Semana</t>
+  </si>
+  <si>
+    <t>Showweekends</t>
+  </si>
+  <si>
+    <t>Mostrar Marcas de fin de semana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CUANDO ESTA ACTIVO, MUESTRA LOS DIAS QUE TIENEN MARCAS REGISTRADAS EN FIN DE SEMANA, TENGA O NO TENGA TURNO, POR PERSONA, DENTRO DEL RANGO DE FECHAS CONSULTADO Y SIEMPRE Y CUANDO NO SEA FERIADO. </t>
+  </si>
+  <si>
+    <t>CUANDO ESTA ACTIVO, MUESTRA LOS FERIADOS QUE TIENEN MARCAS REGISTRADAS PARA LA PERSONA, EN EL RANGO DE FECHAS CONSULTADO. SI FUERA UN DIA SIN TURNO ASIGNADO, ESTE PARAMETRO (ShowHoliday) TIENE PRIORIDAD SOBRE EL EL PARAMETRO "ShowNoTurn" Y "Showweekends". EN ESTE CASO SI SE TIENE MAS DE UNA MARCA, SE TOMA LA PRIMERA Y ULTIMA MARCA DEL DIA Y SE CALCULA EL TIEMPO ENTRE AMBOS COLOCANDO DICHO VALOR EN LAS COLUMNAS DE HORAS EFECTIVAS Y DE PERMANENCIA DEL REPORTE, SI SOLO TIENE UNA MARCA EN EL DIA, SOLO SE MUESTRA EL DIA SIN CALCULOS, COMO ES FERIADO Y NO TIENE TURNO ASIGNADO ENTONCES SE COLOCA EN COLUMNA HORARIO DEL REPORTE: "FERIADO" Y TANTO EN HORA DE INICIO Y DE FIN DEL HORARIO EL VALOR "--". SI TUVIERA TURNO ASIGNADO, ESTE DIA DEBE MANEJARSE Y CALCULARSE COMO CUALQUIER DIA CON TURNO ASIGNADO, PERO EN COLUMNA DE HORARIO COLOCAL AL COSTADO DEL HORARIO EL SIGUIENTE TEXTO "(FER)".</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>*NO USADO*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 30=30 MINUTOS. EN EL EJEMPLO DE FABRICIO DEL REPORTE DEMO, SI FUERA 30, EL CALCULO HUBIERA SIDO 00:50 Y NO 01:20 EN HE PARA LA SALIDA</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">*NO USADO* </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">30=30 MINUTOS. </t>
+    </r>
+  </si>
+  <si>
+    <t>NO VA</t>
   </si>
 </sst>
 </file>
@@ -1949,7 +2018,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2106,6 +2175,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -2411,6 +2486,1338 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
+  <dimension ref="A1:O44"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="3" width="29" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="6" width="8" style="3" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" style="3" customWidth="1"/>
+    <col min="8" max="9" width="8" style="3" customWidth="1"/>
+    <col min="10" max="15" width="11.140625" style="3" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="14"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="I2" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="J2" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="K2" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="L2" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="17"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="19"/>
+      <c r="E3" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I3" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="8"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="19"/>
+      <c r="E4" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I4" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="8"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="19"/>
+      <c r="E5" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I5" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K5" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="8"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="19"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K6" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="L6" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="8"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="21"/>
+      <c r="E7" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="F7" s="10"/>
+      <c r="G7" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="J7" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="K7" s="74" t="s">
+        <v>97</v>
+      </c>
+      <c r="L7" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="11"/>
+    </row>
+    <row r="8" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="19"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="8"/>
+    </row>
+    <row r="9" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="19"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="8"/>
+    </row>
+    <row r="10" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="19"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="8"/>
+    </row>
+    <row r="11" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="21"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="11"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="D12" s="14"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="H12" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="I12" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="J12" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="K12" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="L12" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="M12" s="16"/>
+      <c r="N12" s="16"/>
+      <c r="O12" s="17"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="D13" s="19"/>
+      <c r="E13" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I13" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K13" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="L13" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="8"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14" s="19"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="L14" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
+      <c r="O14" s="8"/>
+    </row>
+    <row r="15" spans="1:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="D15" s="19"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>474</v>
+      </c>
+      <c r="K15" s="7"/>
+      <c r="L15" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M15" s="7"/>
+      <c r="N15" s="7"/>
+      <c r="O15" s="8"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="21"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="J16" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="K16" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="L16" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="M16" s="10"/>
+      <c r="N16" s="10"/>
+      <c r="O16" s="11"/>
+    </row>
+    <row r="17" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" s="19"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M17" s="7"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="8"/>
+    </row>
+    <row r="18" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" s="19"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="7"/>
+      <c r="L18" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
+      <c r="O18" s="8"/>
+    </row>
+    <row r="19" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" s="21"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="11"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="11"/>
+    </row>
+    <row r="20" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" s="14"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M20" s="16"/>
+      <c r="N20" s="16"/>
+      <c r="O20" s="17"/>
+    </row>
+    <row r="21" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" s="19"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="7"/>
+      <c r="L21" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M21" s="7"/>
+      <c r="N21" s="7"/>
+      <c r="O21" s="8"/>
+    </row>
+    <row r="22" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="D22" s="19"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="7"/>
+      <c r="L22" s="7"/>
+      <c r="M22" s="7"/>
+      <c r="N22" s="7"/>
+      <c r="O22" s="8"/>
+    </row>
+    <row r="23" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="D23" s="19"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="7"/>
+      <c r="L23" s="7"/>
+      <c r="M23" s="7"/>
+      <c r="N23" s="7"/>
+      <c r="O23" s="8"/>
+    </row>
+    <row r="24" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="D24" s="21"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="11"/>
+      <c r="K24" s="10"/>
+      <c r="L24" s="10"/>
+      <c r="M24" s="10"/>
+      <c r="N24" s="10"/>
+      <c r="O24" s="11"/>
+    </row>
+    <row r="25" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="D25" s="14"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="16"/>
+      <c r="I25" s="16"/>
+      <c r="J25" s="17"/>
+      <c r="K25" s="16"/>
+      <c r="L25" s="16"/>
+      <c r="M25" s="16"/>
+      <c r="N25" s="16"/>
+      <c r="O25" s="17"/>
+    </row>
+    <row r="26" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="C26" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="D26" s="19"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="7"/>
+      <c r="L26" s="7"/>
+      <c r="M26" s="7"/>
+      <c r="N26" s="7"/>
+      <c r="O26" s="8"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="D27" s="19"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K27" s="7"/>
+      <c r="L27" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M27" s="7"/>
+      <c r="N27" s="7"/>
+      <c r="O27" s="8"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A28" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="D28" s="19"/>
+      <c r="E28" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F28" s="7"/>
+      <c r="G28" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J28" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K28" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="L28" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M28" s="7"/>
+      <c r="N28" s="7"/>
+      <c r="O28" s="8"/>
+    </row>
+    <row r="29" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="C29" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="D29" s="19"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="7"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="7"/>
+      <c r="I29" s="7"/>
+      <c r="J29" s="8"/>
+      <c r="K29" s="7"/>
+      <c r="L29" s="7"/>
+      <c r="M29" s="7"/>
+      <c r="N29" s="7"/>
+      <c r="O29" s="8"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A30" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="D30" s="19"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J30" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K30" s="7"/>
+      <c r="L30" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M30" s="7"/>
+      <c r="N30" s="7"/>
+      <c r="O30" s="8"/>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="C31" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="D31" s="19"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J31" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K31" s="7"/>
+      <c r="L31" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M31" s="7"/>
+      <c r="N31" s="7"/>
+      <c r="O31" s="8"/>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B32" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="C32" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="D32" s="19"/>
+      <c r="E32" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F32" s="7"/>
+      <c r="G32" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I32" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J32" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K32" s="7"/>
+      <c r="L32" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M32" s="7"/>
+      <c r="N32" s="7"/>
+      <c r="O32" s="8"/>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A33" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="C33" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="D33" s="19"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="7"/>
+      <c r="G33" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J33" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K33" s="7"/>
+      <c r="L33" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M33" s="7"/>
+      <c r="N33" s="7"/>
+      <c r="O33" s="8"/>
+    </row>
+    <row r="34" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B34" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="C34" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="D34" s="19"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="8"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="7"/>
+      <c r="J34" s="8"/>
+      <c r="K34" s="7"/>
+      <c r="L34" s="7"/>
+      <c r="M34" s="7"/>
+      <c r="N34" s="7"/>
+      <c r="O34" s="8"/>
+    </row>
+    <row r="35" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B35" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="C35" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="D35" s="19"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="7"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="7"/>
+      <c r="L35" s="7"/>
+      <c r="M35" s="7"/>
+      <c r="N35" s="7"/>
+      <c r="O35" s="8"/>
+    </row>
+    <row r="36" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B36" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="C36" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="D36" s="19"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="7"/>
+      <c r="J36" s="8"/>
+      <c r="K36" s="7"/>
+      <c r="L36" s="7"/>
+      <c r="M36" s="7"/>
+      <c r="N36" s="7"/>
+      <c r="O36" s="8"/>
+    </row>
+    <row r="37" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B37" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C37" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D37" s="21"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="11"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="10"/>
+      <c r="J37" s="11"/>
+      <c r="K37" s="10"/>
+      <c r="L37" s="10"/>
+      <c r="M37" s="10"/>
+      <c r="N37" s="10"/>
+      <c r="O37" s="11"/>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A38" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="D38" s="14"/>
+      <c r="E38" s="15"/>
+      <c r="F38" s="16"/>
+      <c r="G38" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="H38" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="I38" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="J38" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="K38" s="16"/>
+      <c r="L38" s="16"/>
+      <c r="M38" s="16"/>
+      <c r="N38" s="16"/>
+      <c r="O38" s="17"/>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A39" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B39" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="C39" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="D39" s="19"/>
+      <c r="E39" s="6"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I39" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J39" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K39" s="7"/>
+      <c r="L39" s="7"/>
+      <c r="M39" s="7"/>
+      <c r="N39" s="7"/>
+      <c r="O39" s="8"/>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A40" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B40" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="C40" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="D40" s="19"/>
+      <c r="E40" s="6"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I40" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J40" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K40" s="7"/>
+      <c r="L40" s="7"/>
+      <c r="M40" s="7"/>
+      <c r="N40" s="7"/>
+      <c r="O40" s="8"/>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A41" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C41" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="D41" s="19"/>
+      <c r="E41" s="6"/>
+      <c r="F41" s="7"/>
+      <c r="G41" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H41" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I41" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J41" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K41" s="7"/>
+      <c r="L41" s="7"/>
+      <c r="M41" s="7"/>
+      <c r="N41" s="7"/>
+      <c r="O41" s="8"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A42" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="B42" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C42" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="D42" s="19"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="7"/>
+      <c r="G42" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H42" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I42" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J42" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K42" s="7"/>
+      <c r="L42" s="7"/>
+      <c r="M42" s="7"/>
+      <c r="N42" s="7"/>
+      <c r="O42" s="8"/>
+    </row>
+    <row r="43" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="B43" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="C43" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="D43" s="21"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="11"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="11"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="10"/>
+      <c r="M43" s="10"/>
+      <c r="N43" s="10"/>
+      <c r="O43" s="11"/>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="B44" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="C44" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="D44" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="E44" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="F44" s="26"/>
+      <c r="G44" s="27" t="s">
+        <v>92</v>
+      </c>
+      <c r="H44" s="26" t="s">
+        <v>92</v>
+      </c>
+      <c r="I44" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="J44" s="27" t="s">
+        <v>92</v>
+      </c>
+      <c r="K44" s="26"/>
+      <c r="L44" s="26"/>
+      <c r="M44" s="26"/>
+      <c r="N44" s="26"/>
+      <c r="O44" s="27"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:O44">
+    <filterColumn colId="9">
+      <filters>
+        <filter val="SI"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="224" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:N44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3628,12 +5035,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F246"/>
+  <dimension ref="A1:G247"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" style="28" customWidth="1"/>
@@ -3897,12 +5304,12 @@
         <v>288</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="30" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="30" t="s">
         <v>102</v>
       </c>
@@ -3910,12 +5317,12 @@
         <v>101</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="30" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B36" s="28" t="s">
         <v>103</v>
       </c>
@@ -3926,7 +5333,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B37" s="28" t="s">
         <v>104</v>
       </c>
@@ -3937,7 +5344,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B38" s="28" t="s">
         <v>105</v>
       </c>
@@ -3948,12 +5355,12 @@
         <v>203</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="30" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="48" t="s">
         <v>103</v>
       </c>
@@ -3973,7 +5380,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="51" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A41" s="51" t="s">
         <v>107</v>
       </c>
@@ -3992,8 +5399,11 @@
       <c r="F41" s="52" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" ht="51" x14ac:dyDescent="0.25">
+      <c r="G41" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A42" s="42" t="s">
         <v>111</v>
       </c>
@@ -4012,8 +5422,11 @@
       <c r="F42" s="43" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="G42" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A43" s="42" t="s">
         <v>112</v>
       </c>
@@ -4032,8 +5445,11 @@
       <c r="F43" s="43" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" ht="51" x14ac:dyDescent="0.25">
+      <c r="G43" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="42" t="s">
         <v>113</v>
       </c>
@@ -4050,10 +5466,13 @@
         <v>158</v>
       </c>
       <c r="F44" s="43" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
+        <v>472</v>
+      </c>
+      <c r="G44" s="30" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A45" s="42" t="s">
         <v>116</v>
       </c>
@@ -4072,8 +5491,11 @@
       <c r="F45" s="43" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="G45" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="42" t="s">
         <v>117</v>
       </c>
@@ -4090,10 +5512,13 @@
         <v>160</v>
       </c>
       <c r="F46" s="43" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="89.25" x14ac:dyDescent="0.25">
+        <v>473</v>
+      </c>
+      <c r="G46" s="30" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A47" s="42" t="s">
         <v>136</v>
       </c>
@@ -4112,8 +5537,11 @@
       <c r="F47" s="43" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="G47" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A48" s="42" t="s">
         <v>132</v>
       </c>
@@ -4132,8 +5560,11 @@
       <c r="F48" s="43" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" ht="89.25" x14ac:dyDescent="0.25">
+      <c r="G48" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A49" s="42" t="s">
         <v>137</v>
       </c>
@@ -4152,8 +5583,11 @@
       <c r="F49" s="43" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G49" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="53" t="s">
         <v>133</v>
       </c>
@@ -4172,8 +5606,11 @@
       <c r="F50" s="54" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" ht="178.5" x14ac:dyDescent="0.25">
+      <c r="G50" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="191.25" x14ac:dyDescent="0.25">
       <c r="A51" s="38" t="s">
         <v>118</v>
       </c>
@@ -4192,8 +5629,11 @@
       <c r="F51" s="41" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G51" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="42" t="s">
         <v>119</v>
       </c>
@@ -4212,8 +5652,11 @@
       <c r="F52" s="43" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" ht="178.5" x14ac:dyDescent="0.25">
+      <c r="G52" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="178.5" x14ac:dyDescent="0.25">
       <c r="A53" s="42" t="s">
         <v>121</v>
       </c>
@@ -4232,48 +5675,57 @@
       <c r="F53" s="41" t="s">
         <v>431</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A54" s="42" t="s">
+      <c r="G53" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="53" t="s">
         <v>122</v>
       </c>
-      <c r="B54" s="32" t="s">
+      <c r="B54" s="34" t="s">
         <v>109</v>
       </c>
-      <c r="C54" s="32">
+      <c r="C54" s="34">
         <v>44</v>
       </c>
-      <c r="D54" s="33" t="s">
+      <c r="D54" s="35" t="s">
         <v>189</v>
       </c>
-      <c r="E54" s="33" t="s">
+      <c r="E54" s="35" t="s">
         <v>149</v>
       </c>
-      <c r="F54" s="43" t="s">
+      <c r="F54" s="54" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" ht="51" x14ac:dyDescent="0.25">
-      <c r="A55" s="42" t="s">
+      <c r="G54" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+      <c r="A55" s="38" t="s">
         <v>127</v>
       </c>
-      <c r="B55" s="32" t="s">
+      <c r="B55" s="39" t="s">
         <v>109</v>
       </c>
-      <c r="C55" s="32">
+      <c r="C55" s="39">
         <v>1</v>
       </c>
-      <c r="D55" s="33" t="s">
+      <c r="D55" s="40" t="s">
         <v>191</v>
       </c>
-      <c r="E55" s="33" t="s">
+      <c r="E55" s="40" t="s">
         <v>167</v>
       </c>
-      <c r="F55" s="43" t="s">
+      <c r="F55" s="41" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="G55" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A56" s="42" t="s">
         <v>125</v>
       </c>
@@ -4292,8 +5744,11 @@
       <c r="F56" s="43" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" ht="51" x14ac:dyDescent="0.25">
+      <c r="G56" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A57" s="42" t="s">
         <v>126</v>
       </c>
@@ -4312,8 +5767,11 @@
       <c r="F57" s="43" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G57" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="44" t="s">
         <v>124</v>
       </c>
@@ -4332,8 +5790,11 @@
       <c r="F58" s="47" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" ht="153" x14ac:dyDescent="0.25">
+      <c r="G58" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="153" x14ac:dyDescent="0.25">
       <c r="A59" s="51" t="s">
         <v>138</v>
       </c>
@@ -4352,8 +5813,11 @@
       <c r="F59" s="52" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" ht="51" x14ac:dyDescent="0.25">
+      <c r="G59" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A60" s="42" t="s">
         <v>143</v>
       </c>
@@ -4372,8 +5836,11 @@
       <c r="F60" s="43" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" ht="90" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G60" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="90" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="44" t="s">
         <v>142</v>
       </c>
@@ -4392,8 +5859,11 @@
       <c r="F61" s="47" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" ht="216.75" x14ac:dyDescent="0.25">
+      <c r="G61" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="216.75" x14ac:dyDescent="0.25">
       <c r="A62" s="38" t="s">
         <v>139</v>
       </c>
@@ -4407,13 +5877,16 @@
         <v>195</v>
       </c>
       <c r="E62" s="40" t="s">
-        <v>175</v>
+        <v>471</v>
       </c>
       <c r="F62" s="41" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" ht="51" x14ac:dyDescent="0.25">
+      <c r="G62" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A63" s="42" t="s">
         <v>140</v>
       </c>
@@ -4432,8 +5905,11 @@
       <c r="F63" s="43" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" ht="90" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G63" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" ht="90" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="53" t="s">
         <v>141</v>
       </c>
@@ -4452,8 +5928,2687 @@
       <c r="F64" s="54" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+      <c r="G64" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+      <c r="A65" s="38" t="s">
+        <v>468</v>
+      </c>
+      <c r="B65" s="39" t="s">
+        <v>109</v>
+      </c>
+      <c r="C65" s="39"/>
+      <c r="D65" s="40" t="s">
+        <v>469</v>
+      </c>
+      <c r="E65" s="40" t="s">
+        <v>470</v>
+      </c>
+      <c r="F65" s="41" t="s">
+        <v>110</v>
+      </c>
+      <c r="G65" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="114.75" x14ac:dyDescent="0.25">
+      <c r="A66" s="42" t="s">
+        <v>172</v>
+      </c>
+      <c r="B66" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C66" s="32">
+        <v>1</v>
+      </c>
+      <c r="D66" s="33" t="s">
+        <v>466</v>
+      </c>
+      <c r="E66" s="33" t="s">
+        <v>439</v>
+      </c>
+      <c r="F66" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="G66" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" ht="115.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="44" t="s">
+        <v>173</v>
+      </c>
+      <c r="B67" s="45" t="s">
+        <v>109</v>
+      </c>
+      <c r="C67" s="45" t="s">
+        <v>174</v>
+      </c>
+      <c r="D67" s="46" t="s">
+        <v>467</v>
+      </c>
+      <c r="E67" s="46" t="s">
+        <v>440</v>
+      </c>
+      <c r="F67" s="47" t="s">
+        <v>416</v>
+      </c>
+      <c r="G67" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A69" s="30" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B70" s="28" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71" s="30" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A72" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="B72" s="28" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A73" s="30" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B74" s="28" t="s">
+        <v>205</v>
+      </c>
+      <c r="C74" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D74" s="28" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B75" s="28" t="s">
+        <v>206</v>
+      </c>
+      <c r="C75" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D75" s="28" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B76" s="28" t="s">
+        <v>207</v>
+      </c>
+      <c r="C76" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D76" s="28" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B77" s="28" t="s">
+        <v>208</v>
+      </c>
+      <c r="C77" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D77" s="29" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B78" s="28" t="s">
+        <v>209</v>
+      </c>
+      <c r="C78" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D78" s="29" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B79" s="28" t="s">
+        <v>210</v>
+      </c>
+      <c r="C79" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D79" s="56" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B80" s="28" t="s">
+        <v>211</v>
+      </c>
+      <c r="C80" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D80" s="56" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A81" s="30" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="28"/>
+      <c r="B82" s="28" t="s">
+        <v>219</v>
+      </c>
+      <c r="C82" s="28"/>
+      <c r="G82" s="28"/>
+    </row>
+    <row r="83" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="28"/>
+      <c r="B83" s="28" t="s">
+        <v>218</v>
+      </c>
+      <c r="C83" s="28"/>
+      <c r="G83" s="28"/>
+    </row>
+    <row r="84" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="28"/>
+      <c r="B84" s="28" t="s">
+        <v>220</v>
+      </c>
+      <c r="C84" s="28"/>
+      <c r="G84" s="28"/>
+    </row>
+    <row r="85" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="28"/>
+      <c r="B85" s="58"/>
+      <c r="C85" s="28"/>
+      <c r="G85" s="28"/>
+    </row>
+    <row r="86" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="30" t="s">
+        <v>285</v>
+      </c>
+      <c r="B86" s="28"/>
+      <c r="C86" s="28"/>
+      <c r="G86" s="28"/>
+    </row>
+    <row r="87" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="28"/>
+      <c r="B87" s="28" t="s">
+        <v>222</v>
+      </c>
+      <c r="C87" s="28"/>
+      <c r="G87" s="28"/>
+    </row>
+    <row r="88" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A88" s="30" t="s">
+        <v>100</v>
+      </c>
+      <c r="B88" s="28"/>
+      <c r="C88" s="28"/>
+      <c r="G88" s="28"/>
+    </row>
+    <row r="89" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="B89" s="28" t="s">
+        <v>256</v>
+      </c>
+      <c r="C89" s="28"/>
+      <c r="G89" s="28"/>
+    </row>
+    <row r="90" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="B90" s="28"/>
+      <c r="C90" s="28"/>
+      <c r="G90" s="28"/>
+    </row>
+    <row r="91" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="28"/>
+      <c r="B91" s="28" t="s">
+        <v>263</v>
+      </c>
+      <c r="C91" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D91" s="28" t="s">
+        <v>272</v>
+      </c>
+      <c r="G91" s="28"/>
+    </row>
+    <row r="92" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A92" s="28"/>
+      <c r="B92" s="28" t="s">
+        <v>262</v>
+      </c>
+      <c r="C92" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D92" s="28" t="s">
+        <v>273</v>
+      </c>
+      <c r="G92" s="28"/>
+    </row>
+    <row r="93" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A93" s="28"/>
+      <c r="B93" s="28" t="s">
+        <v>261</v>
+      </c>
+      <c r="C93" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D93" s="28" t="s">
+        <v>274</v>
+      </c>
+      <c r="G93" s="28"/>
+    </row>
+    <row r="94" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="28"/>
+      <c r="B94" s="28" t="s">
+        <v>266</v>
+      </c>
+      <c r="C94" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D94" s="28" t="s">
+        <v>275</v>
+      </c>
+      <c r="G94" s="28"/>
+    </row>
+    <row r="95" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="28"/>
+      <c r="B95" s="28" t="s">
+        <v>267</v>
+      </c>
+      <c r="C95" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D95" s="28" t="s">
+        <v>276</v>
+      </c>
+      <c r="G95" s="28"/>
+    </row>
+    <row r="96" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="28"/>
+      <c r="B96" s="28" t="s">
+        <v>268</v>
+      </c>
+      <c r="C96" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D96" s="28" t="s">
+        <v>277</v>
+      </c>
+      <c r="G96" s="28"/>
+    </row>
+    <row r="97" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="28"/>
+      <c r="B97" s="28" t="s">
+        <v>269</v>
+      </c>
+      <c r="C97" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D97" s="28" t="s">
+        <v>278</v>
+      </c>
+      <c r="G97" s="28"/>
+    </row>
+    <row r="98" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="28"/>
+      <c r="B98" s="28" t="s">
+        <v>270</v>
+      </c>
+      <c r="C98" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D98" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="G98" s="28"/>
+    </row>
+    <row r="99" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A99" s="28"/>
+      <c r="B99" s="28" t="s">
+        <v>271</v>
+      </c>
+      <c r="C99" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D99" s="28" t="s">
+        <v>279</v>
+      </c>
+      <c r="G99" s="28"/>
+    </row>
+    <row r="100" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A100" s="30" t="s">
+        <v>217</v>
+      </c>
+      <c r="B100" s="28"/>
+      <c r="C100" s="28"/>
+      <c r="G100" s="28"/>
+    </row>
+    <row r="101" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="28"/>
+      <c r="B101" s="28" t="s">
+        <v>259</v>
+      </c>
+      <c r="C101" s="28"/>
+      <c r="G101" s="28"/>
+    </row>
+    <row r="102" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="28"/>
+      <c r="B102" s="28" t="s">
+        <v>223</v>
+      </c>
+      <c r="C102" s="28"/>
+      <c r="G102" s="28"/>
+    </row>
+    <row r="103" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="28"/>
+      <c r="B103" s="28" t="s">
+        <v>224</v>
+      </c>
+      <c r="C103" s="28"/>
+      <c r="G103" s="28"/>
+    </row>
+    <row r="104" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="28"/>
+      <c r="B104" s="28" t="s">
+        <v>260</v>
+      </c>
+      <c r="C104" s="28"/>
+      <c r="G104" s="28"/>
+    </row>
+    <row r="105" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="28"/>
+      <c r="B105" s="28" t="s">
+        <v>225</v>
+      </c>
+      <c r="C105" s="28"/>
+      <c r="G105" s="28"/>
+    </row>
+    <row r="106" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="28"/>
+      <c r="B106" s="28" t="s">
+        <v>226</v>
+      </c>
+      <c r="C106" s="28"/>
+      <c r="G106" s="28"/>
+    </row>
+    <row r="107" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A107" s="28"/>
+      <c r="B107" s="28" t="s">
+        <v>227</v>
+      </c>
+      <c r="C107" s="28"/>
+      <c r="G107" s="28"/>
+    </row>
+    <row r="108" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A108" s="28"/>
+      <c r="B108" s="28" t="s">
+        <v>281</v>
+      </c>
+      <c r="C108" s="28"/>
+      <c r="G108" s="28"/>
+    </row>
+    <row r="109" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A109" s="28"/>
+      <c r="B109" s="28" t="s">
+        <v>319</v>
+      </c>
+      <c r="C109" s="28"/>
+      <c r="G109" s="28"/>
+    </row>
+    <row r="110" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A110" s="28"/>
+      <c r="B110" s="28" t="s">
+        <v>320</v>
+      </c>
+      <c r="C110" s="28"/>
+      <c r="G110" s="28"/>
+    </row>
+    <row r="111" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A111" s="30" t="s">
+        <v>228</v>
+      </c>
+      <c r="B111" s="28"/>
+      <c r="C111" s="28"/>
+      <c r="G111" s="28"/>
+    </row>
+    <row r="112" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A112" s="28"/>
+      <c r="B112" s="28" t="s">
+        <v>257</v>
+      </c>
+      <c r="C112" s="28"/>
+      <c r="G112" s="28"/>
+    </row>
+    <row r="113" spans="1:7" s="29" customFormat="1" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A113" s="28"/>
+      <c r="B113" s="31" t="s">
+        <v>229</v>
+      </c>
+      <c r="C113" s="59" t="s">
+        <v>236</v>
+      </c>
+      <c r="D113" s="59" t="s">
+        <v>251</v>
+      </c>
+      <c r="G113" s="28"/>
+    </row>
+    <row r="114" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="28"/>
+      <c r="B114" s="32" t="s">
+        <v>230</v>
+      </c>
+      <c r="C114" s="32" t="s">
+        <v>231</v>
+      </c>
+      <c r="D114" s="60" t="s">
+        <v>232</v>
+      </c>
+      <c r="G114" s="28"/>
+    </row>
+    <row r="115" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="28"/>
+      <c r="B115" s="32" t="s">
+        <v>233</v>
+      </c>
+      <c r="C115" s="32" t="s">
+        <v>234</v>
+      </c>
+      <c r="D115" s="60" t="s">
+        <v>238</v>
+      </c>
+      <c r="G115" s="28"/>
+    </row>
+    <row r="116" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A116" s="28"/>
+      <c r="B116" s="61" t="s">
+        <v>235</v>
+      </c>
+      <c r="C116" s="32" t="s">
+        <v>237</v>
+      </c>
+      <c r="D116" s="60" t="s">
+        <v>242</v>
+      </c>
+      <c r="G116" s="28"/>
+    </row>
+    <row r="117" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A117" s="28"/>
+      <c r="B117" s="61" t="s">
+        <v>239</v>
+      </c>
+      <c r="C117" s="32" t="s">
+        <v>240</v>
+      </c>
+      <c r="D117" s="60" t="s">
+        <v>241</v>
+      </c>
+      <c r="G117" s="28"/>
+    </row>
+    <row r="118" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A118" s="28"/>
+      <c r="B118" s="32" t="s">
+        <v>243</v>
+      </c>
+      <c r="C118" s="32" t="s">
+        <v>244</v>
+      </c>
+      <c r="D118" s="60" t="s">
+        <v>241</v>
+      </c>
+      <c r="G118" s="28"/>
+    </row>
+    <row r="119" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A119" s="28"/>
+      <c r="B119" s="32" t="s">
+        <v>245</v>
+      </c>
+      <c r="C119" s="32" t="s">
+        <v>246</v>
+      </c>
+      <c r="D119" s="60" t="s">
+        <v>252</v>
+      </c>
+      <c r="G119" s="28"/>
+    </row>
+    <row r="120" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A120" s="28"/>
+      <c r="B120" s="32" t="s">
+        <v>247</v>
+      </c>
+      <c r="C120" s="32" t="s">
+        <v>250</v>
+      </c>
+      <c r="D120" s="60" t="s">
+        <v>241</v>
+      </c>
+      <c r="G120" s="28"/>
+    </row>
+    <row r="121" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A121" s="28"/>
+      <c r="B121" s="32" t="s">
+        <v>248</v>
+      </c>
+      <c r="C121" s="32" t="s">
+        <v>249</v>
+      </c>
+      <c r="D121" s="60" t="s">
+        <v>241</v>
+      </c>
+      <c r="G121" s="28"/>
+    </row>
+    <row r="122" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A122" s="28"/>
+      <c r="B122" s="56" t="s">
+        <v>258</v>
+      </c>
+      <c r="G122" s="28"/>
+    </row>
+    <row r="123" spans="1:7" s="29" customFormat="1" ht="51" x14ac:dyDescent="0.25">
+      <c r="A123" s="28"/>
+      <c r="B123" s="32" t="s">
+        <v>253</v>
+      </c>
+      <c r="C123" s="61" t="s">
+        <v>254</v>
+      </c>
+      <c r="D123" s="33" t="s">
+        <v>255</v>
+      </c>
+      <c r="G123" s="28"/>
+    </row>
+    <row r="125" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="30" t="s">
+        <v>321</v>
+      </c>
+      <c r="B125" s="28"/>
+      <c r="C125" s="28"/>
+      <c r="G125" s="28"/>
+    </row>
+    <row r="126" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A126" s="28"/>
+      <c r="B126" s="28" t="s">
+        <v>354</v>
+      </c>
+      <c r="C126" s="28"/>
+      <c r="G126" s="28"/>
+    </row>
+    <row r="127" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A127" s="30" t="s">
+        <v>100</v>
+      </c>
+      <c r="B127" s="28"/>
+      <c r="C127" s="28"/>
+      <c r="G127" s="28"/>
+    </row>
+    <row r="128" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A128" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="B128" s="28" t="s">
+        <v>322</v>
+      </c>
+      <c r="C128" s="28"/>
+      <c r="G128" s="28"/>
+    </row>
+    <row r="129" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A129" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="B129" s="28"/>
+      <c r="C129" s="28"/>
+      <c r="G129" s="28"/>
+    </row>
+    <row r="130" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A130" s="28"/>
+      <c r="B130" s="28" t="s">
+        <v>323</v>
+      </c>
+      <c r="C130" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D130" s="56" t="s">
+        <v>339</v>
+      </c>
+      <c r="G130" s="28"/>
+    </row>
+    <row r="131" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A131" s="28"/>
+      <c r="B131" s="28" t="s">
+        <v>324</v>
+      </c>
+      <c r="C131" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D131" s="56" t="s">
+        <v>340</v>
+      </c>
+      <c r="G131" s="28"/>
+    </row>
+    <row r="132" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A132" s="28"/>
+      <c r="B132" s="28" t="s">
+        <v>325</v>
+      </c>
+      <c r="C132" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D132" s="56" t="s">
+        <v>341</v>
+      </c>
+      <c r="G132" s="28"/>
+    </row>
+    <row r="133" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A133" s="28"/>
+      <c r="B133" s="28" t="s">
+        <v>326</v>
+      </c>
+      <c r="C133" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D133" s="56" t="s">
+        <v>342</v>
+      </c>
+      <c r="G133" s="28"/>
+    </row>
+    <row r="134" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A134" s="28"/>
+      <c r="B134" s="28" t="s">
+        <v>327</v>
+      </c>
+      <c r="C134" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D134" s="56" t="s">
+        <v>343</v>
+      </c>
+      <c r="G134" s="28"/>
+    </row>
+    <row r="135" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A135" s="28"/>
+      <c r="B135" s="28" t="s">
+        <v>328</v>
+      </c>
+      <c r="C135" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D135" s="56" t="s">
+        <v>343</v>
+      </c>
+      <c r="G135" s="28"/>
+    </row>
+    <row r="136" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A136" s="28"/>
+      <c r="B136" s="28" t="s">
+        <v>329</v>
+      </c>
+      <c r="C136" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D136" s="56" t="s">
+        <v>344</v>
+      </c>
+      <c r="G136" s="28"/>
+    </row>
+    <row r="137" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A137" s="28"/>
+      <c r="B137" s="28" t="s">
+        <v>330</v>
+      </c>
+      <c r="C137" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D137" s="56" t="s">
+        <v>345</v>
+      </c>
+      <c r="G137" s="28"/>
+    </row>
+    <row r="138" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A138" s="28"/>
+      <c r="B138" s="28" t="s">
+        <v>331</v>
+      </c>
+      <c r="C138" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D138" s="56" t="s">
+        <v>346</v>
+      </c>
+      <c r="G138" s="28"/>
+    </row>
+    <row r="139" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="28"/>
+      <c r="B139" s="28" t="s">
+        <v>332</v>
+      </c>
+      <c r="C139" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D139" s="56" t="s">
+        <v>347</v>
+      </c>
+      <c r="G139" s="28"/>
+    </row>
+    <row r="140" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A140" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="B140" s="28" t="s">
+        <v>333</v>
+      </c>
+      <c r="C140" s="28"/>
+      <c r="D140" s="56"/>
+      <c r="G140" s="28"/>
+    </row>
+    <row r="141" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A141" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="B141" s="28"/>
+      <c r="C141" s="28"/>
+      <c r="D141" s="56"/>
+      <c r="G141" s="28"/>
+    </row>
+    <row r="142" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A142" s="28"/>
+      <c r="B142" s="28" t="s">
+        <v>263</v>
+      </c>
+      <c r="C142" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D142" s="56" t="s">
+        <v>348</v>
+      </c>
+      <c r="G142" s="28"/>
+    </row>
+    <row r="143" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A143" s="28"/>
+      <c r="B143" s="28" t="s">
+        <v>334</v>
+      </c>
+      <c r="C143" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D143" s="56" t="s">
+        <v>352</v>
+      </c>
+      <c r="G143" s="28"/>
+    </row>
+    <row r="144" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A144" s="28"/>
+      <c r="B144" s="28" t="s">
+        <v>335</v>
+      </c>
+      <c r="C144" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D144" s="56" t="s">
+        <v>353</v>
+      </c>
+      <c r="G144" s="28"/>
+    </row>
+    <row r="145" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A145" s="28"/>
+      <c r="B145" s="28" t="s">
+        <v>336</v>
+      </c>
+      <c r="C145" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D145" s="56" t="s">
+        <v>349</v>
+      </c>
+      <c r="G145" s="28"/>
+    </row>
+    <row r="146" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A146" s="28"/>
+      <c r="B146" s="28" t="s">
+        <v>337</v>
+      </c>
+      <c r="C146" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D146" s="56" t="s">
+        <v>350</v>
+      </c>
+      <c r="G146" s="28"/>
+    </row>
+    <row r="147" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A147" s="28"/>
+      <c r="B147" s="28" t="s">
+        <v>338</v>
+      </c>
+      <c r="C147" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D147" s="56" t="s">
+        <v>351</v>
+      </c>
+      <c r="G147" s="28"/>
+    </row>
+    <row r="148" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A148" s="30" t="s">
+        <v>217</v>
+      </c>
+      <c r="B148" s="28"/>
+      <c r="C148" s="28"/>
+      <c r="D148" s="56"/>
+      <c r="G148" s="28"/>
+    </row>
+    <row r="149" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A149" s="28"/>
+      <c r="B149" s="28" t="s">
+        <v>355</v>
+      </c>
+      <c r="C149" s="28"/>
+      <c r="G149" s="28"/>
+    </row>
+    <row r="150" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A150" s="28"/>
+      <c r="B150" s="28" t="s">
+        <v>356</v>
+      </c>
+      <c r="C150" s="28"/>
+      <c r="G150" s="28"/>
+    </row>
+    <row r="151" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A151" s="28"/>
+      <c r="B151" s="28" t="s">
+        <v>357</v>
+      </c>
+      <c r="C151" s="28"/>
+      <c r="G151" s="28"/>
+    </row>
+    <row r="152" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A152" s="28"/>
+      <c r="B152" s="28" t="s">
+        <v>358</v>
+      </c>
+      <c r="C152" s="28"/>
+      <c r="G152" s="28"/>
+    </row>
+    <row r="153" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A153" s="28"/>
+      <c r="B153" s="28" t="s">
+        <v>359</v>
+      </c>
+      <c r="C153" s="28"/>
+      <c r="G153" s="28"/>
+    </row>
+    <row r="154" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A154" s="28"/>
+      <c r="B154" s="28" t="s">
+        <v>374</v>
+      </c>
+      <c r="C154" s="28"/>
+      <c r="G154" s="28"/>
+    </row>
+    <row r="155" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A155" s="28"/>
+      <c r="B155" s="28" t="s">
+        <v>360</v>
+      </c>
+      <c r="C155" s="28"/>
+      <c r="G155" s="28"/>
+    </row>
+    <row r="156" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A156" s="28"/>
+      <c r="B156" s="28" t="s">
+        <v>361</v>
+      </c>
+      <c r="C156" s="28"/>
+      <c r="G156" s="28"/>
+    </row>
+    <row r="157" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A157" s="28"/>
+      <c r="B157" s="28" t="s">
+        <v>368</v>
+      </c>
+      <c r="C157" s="28"/>
+      <c r="G157" s="28"/>
+    </row>
+    <row r="158" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A158" s="28"/>
+      <c r="B158" s="28" t="s">
+        <v>362</v>
+      </c>
+      <c r="C158" s="28"/>
+      <c r="G158" s="28"/>
+    </row>
+    <row r="159" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A159" s="28"/>
+      <c r="B159" s="28" t="s">
+        <v>363</v>
+      </c>
+      <c r="C159" s="28"/>
+      <c r="G159" s="28"/>
+    </row>
+    <row r="160" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A160" s="28"/>
+      <c r="B160" s="28" t="s">
+        <v>364</v>
+      </c>
+      <c r="C160" s="28"/>
+      <c r="G160" s="28"/>
+    </row>
+    <row r="161" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A161" s="28"/>
+      <c r="B161" s="28" t="s">
+        <v>365</v>
+      </c>
+      <c r="C161" s="28"/>
+      <c r="G161" s="28"/>
+    </row>
+    <row r="162" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A162" s="28"/>
+      <c r="B162" s="28" t="s">
+        <v>369</v>
+      </c>
+      <c r="C162" s="28"/>
+      <c r="G162" s="28"/>
+    </row>
+    <row r="163" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A163" s="28"/>
+      <c r="B163" s="28" t="s">
+        <v>370</v>
+      </c>
+      <c r="C163" s="28"/>
+      <c r="G163" s="28"/>
+    </row>
+    <row r="164" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="28"/>
+      <c r="B164" s="28" t="s">
+        <v>371</v>
+      </c>
+      <c r="C164" s="28"/>
+      <c r="G164" s="28"/>
+    </row>
+    <row r="165" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A165" s="28"/>
+      <c r="B165" s="28" t="s">
+        <v>372</v>
+      </c>
+      <c r="C165" s="28"/>
+      <c r="G165" s="28"/>
+    </row>
+    <row r="166" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A166" s="28"/>
+      <c r="B166" s="28" t="s">
+        <v>373</v>
+      </c>
+      <c r="C166" s="28"/>
+      <c r="G166" s="28"/>
+    </row>
+    <row r="167" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A167" s="28"/>
+      <c r="B167" s="28" t="s">
+        <v>366</v>
+      </c>
+      <c r="C167" s="28"/>
+      <c r="G167" s="28"/>
+    </row>
+    <row r="168" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A168" s="28"/>
+      <c r="B168" s="28" t="s">
+        <v>367</v>
+      </c>
+      <c r="C168" s="28"/>
+      <c r="G168" s="28"/>
+    </row>
+    <row r="170" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A170" s="30" t="s">
+        <v>375</v>
+      </c>
+      <c r="B170" s="28"/>
+      <c r="C170" s="28"/>
+      <c r="G170" s="28"/>
+    </row>
+    <row r="171" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A171" s="28"/>
+      <c r="B171" s="28" t="s">
+        <v>376</v>
+      </c>
+      <c r="C171" s="28"/>
+      <c r="G171" s="28"/>
+    </row>
+    <row r="172" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A172" s="28"/>
+      <c r="B172" s="28" t="s">
+        <v>377</v>
+      </c>
+      <c r="C172" s="28"/>
+      <c r="G172" s="28"/>
+    </row>
+    <row r="173" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A173" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="B173" s="28" t="s">
+        <v>394</v>
+      </c>
+      <c r="C173" s="28"/>
+      <c r="G173" s="28"/>
+    </row>
+    <row r="174" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A174" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="B174" s="28"/>
+      <c r="C174" s="28"/>
+      <c r="G174" s="28"/>
+    </row>
+    <row r="175" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A175" s="28"/>
+      <c r="B175" s="28" t="s">
+        <v>378</v>
+      </c>
+      <c r="C175" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D175" s="56" t="s">
+        <v>395</v>
+      </c>
+      <c r="G175" s="28"/>
+    </row>
+    <row r="176" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A176" s="28"/>
+      <c r="B176" s="28" t="s">
+        <v>379</v>
+      </c>
+      <c r="C176" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D176" s="56" t="s">
+        <v>464</v>
+      </c>
+      <c r="G176" s="28"/>
+    </row>
+    <row r="177" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A177" s="28"/>
+      <c r="B177" s="28"/>
+      <c r="C177" s="28"/>
+      <c r="D177" s="56" t="s">
+        <v>396</v>
+      </c>
+      <c r="G177" s="28"/>
+    </row>
+    <row r="178" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A178" s="28"/>
+      <c r="B178" s="28"/>
+      <c r="C178" s="28"/>
+      <c r="D178" s="56" t="s">
+        <v>397</v>
+      </c>
+      <c r="G178" s="28"/>
+    </row>
+    <row r="179" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A179" s="28"/>
+      <c r="B179" s="28" t="s">
+        <v>380</v>
+      </c>
+      <c r="C179" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D179" s="56" t="s">
+        <v>399</v>
+      </c>
+      <c r="G179" s="28"/>
+    </row>
+    <row r="180" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A180" s="28"/>
+      <c r="B180" s="28" t="s">
+        <v>381</v>
+      </c>
+      <c r="C180" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D180" s="56" t="s">
+        <v>398</v>
+      </c>
+      <c r="G180" s="28"/>
+    </row>
+    <row r="181" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A181" s="28"/>
+      <c r="B181" s="28" t="s">
+        <v>382</v>
+      </c>
+      <c r="C181" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D181" s="56" t="s">
+        <v>400</v>
+      </c>
+      <c r="G181" s="28"/>
+    </row>
+    <row r="182" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A182" s="28"/>
+      <c r="B182" s="28" t="s">
+        <v>383</v>
+      </c>
+      <c r="C182" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D182" s="56" t="s">
+        <v>401</v>
+      </c>
+      <c r="G182" s="28"/>
+    </row>
+    <row r="183" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A183" s="28"/>
+      <c r="B183" s="28" t="s">
+        <v>384</v>
+      </c>
+      <c r="C183" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D183" s="56" t="s">
+        <v>402</v>
+      </c>
+      <c r="G183" s="28"/>
+    </row>
+    <row r="184" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A184" s="28"/>
+      <c r="B184" s="28" t="s">
+        <v>385</v>
+      </c>
+      <c r="C184" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D184" s="56" t="s">
+        <v>402</v>
+      </c>
+      <c r="G184" s="28"/>
+    </row>
+    <row r="185" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A185" s="28"/>
+      <c r="B185" s="28"/>
+      <c r="C185" s="28"/>
+      <c r="D185" s="56" t="s">
+        <v>404</v>
+      </c>
+      <c r="G185" s="28"/>
+    </row>
+    <row r="186" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A186" s="28"/>
+      <c r="B186" s="28"/>
+      <c r="C186" s="28"/>
+      <c r="D186" s="56" t="s">
+        <v>409</v>
+      </c>
+      <c r="G186" s="28"/>
+    </row>
+    <row r="187" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A187" s="28"/>
+      <c r="B187" s="62" t="s">
+        <v>386</v>
+      </c>
+      <c r="C187" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D187" s="56" t="s">
+        <v>407</v>
+      </c>
+      <c r="G187" s="28"/>
+    </row>
+    <row r="188" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A188" s="28"/>
+      <c r="B188" s="62" t="s">
+        <v>387</v>
+      </c>
+      <c r="C188" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D188" s="56" t="s">
+        <v>408</v>
+      </c>
+      <c r="G188" s="28"/>
+    </row>
+    <row r="189" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="28"/>
+      <c r="B189" s="62"/>
+      <c r="C189" s="28"/>
+      <c r="D189" s="56" t="s">
+        <v>403</v>
+      </c>
+      <c r="G189" s="28"/>
+    </row>
+    <row r="190" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A190" s="28"/>
+      <c r="B190" s="62"/>
+      <c r="C190" s="28"/>
+      <c r="D190" s="56" t="s">
+        <v>409</v>
+      </c>
+      <c r="G190" s="28"/>
+    </row>
+    <row r="191" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A191" s="28"/>
+      <c r="B191" s="62" t="s">
+        <v>388</v>
+      </c>
+      <c r="C191" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D191" s="56" t="s">
+        <v>405</v>
+      </c>
+      <c r="G191" s="28"/>
+    </row>
+    <row r="192" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A192" s="28"/>
+      <c r="B192" s="62" t="s">
+        <v>389</v>
+      </c>
+      <c r="C192" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D192" s="56" t="s">
+        <v>406</v>
+      </c>
+      <c r="G192" s="28"/>
+    </row>
+    <row r="193" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A193" s="28"/>
+      <c r="B193" s="28" t="s">
+        <v>331</v>
+      </c>
+      <c r="C193" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D193" s="56" t="s">
+        <v>410</v>
+      </c>
+      <c r="G193" s="28"/>
+    </row>
+    <row r="194" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A194" s="28"/>
+      <c r="B194" s="28" t="s">
+        <v>390</v>
+      </c>
+      <c r="C194" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D194" s="56" t="s">
+        <v>402</v>
+      </c>
+      <c r="G194" s="28"/>
+    </row>
+    <row r="195" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A195" s="28"/>
+      <c r="B195" s="28" t="s">
+        <v>391</v>
+      </c>
+      <c r="C195" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D195" s="56" t="s">
+        <v>402</v>
+      </c>
+      <c r="G195" s="28"/>
+    </row>
+    <row r="196" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A196" s="28"/>
+      <c r="B196" s="28" t="s">
+        <v>392</v>
+      </c>
+      <c r="C196" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D196" s="29" t="s">
+        <v>350</v>
+      </c>
+      <c r="G196" s="28"/>
+    </row>
+    <row r="197" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A197" s="28"/>
+      <c r="B197" s="28" t="s">
+        <v>393</v>
+      </c>
+      <c r="C197" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="D197" s="56" t="s">
+        <v>411</v>
+      </c>
+      <c r="G197" s="28"/>
+    </row>
+    <row r="198" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A198" s="30" t="s">
+        <v>217</v>
+      </c>
+      <c r="B198" s="28"/>
+      <c r="C198" s="28"/>
+      <c r="G198" s="28"/>
+    </row>
+    <row r="199" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A199" s="28"/>
+      <c r="B199" s="28" t="s">
+        <v>432</v>
+      </c>
+      <c r="C199" s="28"/>
+      <c r="G199" s="28"/>
+    </row>
+    <row r="200" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A200" s="28"/>
+      <c r="B200" s="28" t="s">
+        <v>412</v>
+      </c>
+      <c r="C200" s="28"/>
+      <c r="G200" s="28"/>
+    </row>
+    <row r="201" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A201" s="28"/>
+      <c r="B201" s="28"/>
+      <c r="C201" s="28" t="s">
+        <v>414</v>
+      </c>
+      <c r="G201" s="28"/>
+    </row>
+    <row r="202" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A202" s="28"/>
+      <c r="B202" s="28"/>
+      <c r="C202" s="28" t="s">
+        <v>415</v>
+      </c>
+      <c r="G202" s="28"/>
+    </row>
+    <row r="203" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A203" s="28"/>
+      <c r="B203" s="28"/>
+      <c r="C203" s="28" t="s">
+        <v>433</v>
+      </c>
+      <c r="G203" s="28"/>
+    </row>
+    <row r="204" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A204" s="28"/>
+      <c r="B204" s="28"/>
+      <c r="C204" s="28" t="s">
+        <v>421</v>
+      </c>
+      <c r="G204" s="28"/>
+    </row>
+    <row r="205" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A205" s="28"/>
+      <c r="B205" s="28"/>
+      <c r="C205" s="28" t="s">
+        <v>434</v>
+      </c>
+      <c r="G205" s="28"/>
+    </row>
+    <row r="206" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A206" s="28"/>
+      <c r="B206" s="28"/>
+      <c r="C206" s="28" t="s">
+        <v>435</v>
+      </c>
+      <c r="G206" s="28"/>
+    </row>
+    <row r="207" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A207" s="28"/>
+      <c r="B207" s="28"/>
+      <c r="C207" s="28" t="s">
+        <v>436</v>
+      </c>
+      <c r="G207" s="28"/>
+    </row>
+    <row r="208" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A208" s="28"/>
+      <c r="B208" s="28"/>
+      <c r="C208" s="28" t="s">
+        <v>417</v>
+      </c>
+      <c r="G208" s="28"/>
+    </row>
+    <row r="209" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A209" s="28"/>
+      <c r="B209" s="28" t="s">
+        <v>413</v>
+      </c>
+      <c r="C209" s="28"/>
+      <c r="G209" s="28"/>
+    </row>
+    <row r="210" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A210" s="28"/>
+      <c r="B210" s="28"/>
+      <c r="C210" s="28" t="s">
+        <v>418</v>
+      </c>
+      <c r="G210" s="28"/>
+    </row>
+    <row r="211" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A211" s="28"/>
+      <c r="B211" s="28"/>
+      <c r="C211" s="28" t="s">
+        <v>449</v>
+      </c>
+      <c r="G211" s="28"/>
+    </row>
+    <row r="212" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A212" s="28"/>
+      <c r="B212" s="28"/>
+      <c r="C212" s="28" t="s">
+        <v>450</v>
+      </c>
+      <c r="G212" s="28"/>
+    </row>
+    <row r="213" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A213" s="28"/>
+      <c r="B213" s="28"/>
+      <c r="C213" s="28" t="s">
+        <v>451</v>
+      </c>
+      <c r="G213" s="28"/>
+    </row>
+    <row r="214" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A214" s="28"/>
+      <c r="B214" s="28"/>
+      <c r="C214" s="28" t="s">
+        <v>452</v>
+      </c>
+      <c r="G214" s="28"/>
+    </row>
+    <row r="215" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A215" s="28"/>
+      <c r="B215" s="28"/>
+      <c r="C215" s="28" t="s">
+        <v>454</v>
+      </c>
+      <c r="G215" s="28"/>
+    </row>
+    <row r="216" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A216" s="28"/>
+      <c r="B216" s="28"/>
+      <c r="C216" s="28" t="s">
+        <v>453</v>
+      </c>
+      <c r="G216" s="28"/>
+    </row>
+    <row r="217" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A217" s="28"/>
+      <c r="B217" s="28"/>
+      <c r="C217" s="58" t="s">
+        <v>455</v>
+      </c>
+      <c r="G217" s="28"/>
+    </row>
+    <row r="218" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A218" s="28"/>
+      <c r="B218" s="28"/>
+      <c r="C218" s="28"/>
+      <c r="D218" s="73" t="s">
+        <v>419</v>
+      </c>
+      <c r="E218" s="73"/>
+      <c r="G218" s="28"/>
+    </row>
+    <row r="219" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A219" s="28"/>
+      <c r="B219" s="28"/>
+      <c r="C219" s="58" t="s">
+        <v>456</v>
+      </c>
+      <c r="D219" s="72"/>
+      <c r="E219" s="72"/>
+      <c r="G219" s="28"/>
+    </row>
+    <row r="220" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A220" s="28"/>
+      <c r="B220" s="28"/>
+      <c r="C220" s="28"/>
+      <c r="D220" s="73" t="s">
+        <v>420</v>
+      </c>
+      <c r="E220" s="73"/>
+      <c r="G220" s="28"/>
+    </row>
+    <row r="221" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A221" s="28"/>
+      <c r="B221" s="28"/>
+      <c r="C221" s="28" t="s">
+        <v>457</v>
+      </c>
+      <c r="G221" s="28"/>
+    </row>
+    <row r="222" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A222" s="28"/>
+      <c r="B222" s="28"/>
+      <c r="C222" s="28" t="s">
+        <v>458</v>
+      </c>
+      <c r="G222" s="28"/>
+    </row>
+    <row r="223" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A223" s="28"/>
+      <c r="B223" s="28"/>
+      <c r="C223" s="28" t="s">
+        <v>459</v>
+      </c>
+      <c r="G223" s="28"/>
+    </row>
+    <row r="224" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A224" s="28"/>
+      <c r="B224" s="28"/>
+      <c r="C224" s="28" t="s">
+        <v>460</v>
+      </c>
+      <c r="G224" s="28"/>
+    </row>
+    <row r="225" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A225" s="28"/>
+      <c r="B225" s="28"/>
+      <c r="C225" s="28" t="s">
+        <v>461</v>
+      </c>
+      <c r="G225" s="28"/>
+    </row>
+    <row r="226" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A226" s="28"/>
+      <c r="B226" s="28"/>
+      <c r="C226" s="28" t="s">
+        <v>462</v>
+      </c>
+      <c r="G226" s="28"/>
+    </row>
+    <row r="227" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A227" s="28"/>
+      <c r="B227" s="28"/>
+      <c r="C227" s="28" t="s">
+        <v>422</v>
+      </c>
+      <c r="G227" s="28"/>
+    </row>
+    <row r="228" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A228" s="28"/>
+      <c r="B228" s="28"/>
+      <c r="C228" s="28" t="s">
+        <v>463</v>
+      </c>
+      <c r="G228" s="28"/>
+    </row>
+    <row r="229" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A229" s="28"/>
+      <c r="B229" s="28"/>
+      <c r="C229" s="28" t="s">
+        <v>423</v>
+      </c>
+      <c r="G229" s="28"/>
+    </row>
+    <row r="230" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A230" s="28"/>
+      <c r="B230" s="28"/>
+      <c r="C230" s="28" t="s">
+        <v>424</v>
+      </c>
+      <c r="G230" s="28"/>
+    </row>
+    <row r="231" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A231" s="28"/>
+      <c r="B231" s="28"/>
+      <c r="C231" s="28" t="s">
+        <v>427</v>
+      </c>
+      <c r="G231" s="28"/>
+    </row>
+    <row r="232" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A232" s="28"/>
+      <c r="B232" s="28"/>
+      <c r="C232" s="28" t="s">
+        <v>426</v>
+      </c>
+      <c r="G232" s="28"/>
+    </row>
+    <row r="233" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A233" s="28"/>
+      <c r="B233" s="28"/>
+      <c r="C233" s="28" t="s">
+        <v>425</v>
+      </c>
+      <c r="G233" s="28"/>
+    </row>
+    <row r="234" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A234" s="28"/>
+      <c r="B234" s="28"/>
+      <c r="C234" s="28" t="s">
+        <v>428</v>
+      </c>
+      <c r="G234" s="28"/>
+    </row>
+    <row r="235" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A235" s="28"/>
+      <c r="B235" s="28"/>
+      <c r="C235" s="28" t="s">
+        <v>429</v>
+      </c>
+      <c r="G235" s="28"/>
+    </row>
+    <row r="236" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A236" s="28"/>
+      <c r="B236" s="28"/>
+      <c r="C236" s="28" t="s">
+        <v>430</v>
+      </c>
+      <c r="G236" s="28"/>
+    </row>
+    <row r="237" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A237" s="28"/>
+      <c r="B237" s="28"/>
+      <c r="C237" s="28" t="s">
+        <v>437</v>
+      </c>
+      <c r="G237" s="28"/>
+    </row>
+    <row r="238" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A238" s="28"/>
+      <c r="B238" s="28"/>
+      <c r="C238" s="28" t="s">
+        <v>438</v>
+      </c>
+      <c r="G238" s="28"/>
+    </row>
+    <row r="239" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A239" s="30" t="s">
+        <v>441</v>
+      </c>
+      <c r="B239" s="28"/>
+      <c r="C239" s="28"/>
+      <c r="G239" s="28"/>
+    </row>
+    <row r="240" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A240" s="28"/>
+      <c r="B240" s="64"/>
+      <c r="C240" s="33" t="s">
+        <v>99</v>
+      </c>
+      <c r="G240" s="28"/>
+    </row>
+    <row r="241" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A241" s="28"/>
+      <c r="B241" s="65"/>
+      <c r="C241" s="33" t="s">
+        <v>442</v>
+      </c>
+      <c r="G241" s="28"/>
+    </row>
+    <row r="242" spans="1:7" s="29" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A242" s="28"/>
+      <c r="B242" s="66"/>
+      <c r="C242" s="33" t="s">
+        <v>443</v>
+      </c>
+      <c r="G242" s="28"/>
+    </row>
+    <row r="243" spans="1:7" s="29" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A243" s="28"/>
+      <c r="B243" s="67"/>
+      <c r="C243" s="33" t="s">
+        <v>444</v>
+      </c>
+      <c r="G243" s="28"/>
+    </row>
+    <row r="244" spans="1:7" s="29" customFormat="1" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A244" s="28"/>
+      <c r="B244" s="68"/>
+      <c r="C244" s="33" t="s">
+        <v>445</v>
+      </c>
+      <c r="G244" s="28"/>
+    </row>
+    <row r="245" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A245" s="28"/>
+      <c r="B245" s="69"/>
+      <c r="C245" s="33" t="s">
+        <v>446</v>
+      </c>
+      <c r="G245" s="28"/>
+    </row>
+    <row r="246" spans="1:7" s="29" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A246" s="28"/>
+      <c r="B246" s="70"/>
+      <c r="C246" s="33" t="s">
+        <v>447</v>
+      </c>
+      <c r="G246" s="28"/>
+    </row>
+    <row r="247" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A247" s="28"/>
+      <c r="B247" s="71"/>
+      <c r="C247" s="33" t="s">
+        <v>448</v>
+      </c>
+      <c r="G247" s="28"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="D218:E218"/>
+    <mergeCell ref="D220:E220"/>
+  </mergeCells>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="57" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G246"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13" style="28" customWidth="1"/>
+    <col min="2" max="3" width="8.85546875" style="28" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" style="29" customWidth="1"/>
+    <col min="5" max="5" width="44.7109375" style="29" customWidth="1"/>
+    <col min="6" max="6" width="33.42578125" style="29" customWidth="1"/>
+    <col min="7" max="16384" width="11.42578125" style="28"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="30" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="56" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="56"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="30" t="s">
+        <v>283</v>
+      </c>
+      <c r="B4" s="56"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="56" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="30" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="B7" s="28" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="30" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B9" s="28" t="s">
+        <v>290</v>
+      </c>
+      <c r="C9" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D9" s="28" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B10" s="28" t="s">
+        <v>291</v>
+      </c>
+      <c r="C10" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D10" s="28" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B11" s="28" t="s">
+        <v>292</v>
+      </c>
+      <c r="C11" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D11" s="28" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B12" s="28" t="s">
+        <v>293</v>
+      </c>
+      <c r="C12" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D12" s="28" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B13" s="28" t="s">
+        <v>294</v>
+      </c>
+      <c r="C13" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D13" s="28" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B14" s="28" t="s">
+        <v>295</v>
+      </c>
+      <c r="C14" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D14" s="28" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B15" s="28" t="s">
+        <v>296</v>
+      </c>
+      <c r="C15" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D15" s="28" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B16" s="28" t="s">
+        <v>297</v>
+      </c>
+      <c r="C16" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D16" s="28" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B17" s="28" t="s">
+        <v>298</v>
+      </c>
+      <c r="C17" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D17" s="28" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="30" t="s">
+        <v>217</v>
+      </c>
+      <c r="C18" s="57"/>
+      <c r="D18" s="28"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="30"/>
+      <c r="B19" s="28" t="s">
+        <v>308</v>
+      </c>
+      <c r="C19" s="57"/>
+      <c r="D19" s="28"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="30"/>
+      <c r="B20" s="28" t="s">
+        <v>310</v>
+      </c>
+      <c r="C20" s="57"/>
+      <c r="D20" s="28"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="30"/>
+      <c r="B21" s="28" t="s">
+        <v>312</v>
+      </c>
+      <c r="C21" s="57"/>
+      <c r="D21" s="28"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="30"/>
+      <c r="B22" s="28" t="s">
+        <v>313</v>
+      </c>
+      <c r="C22" s="57"/>
+      <c r="D22" s="28"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="30"/>
+      <c r="B23" s="28" t="s">
+        <v>309</v>
+      </c>
+      <c r="C23" s="57"/>
+      <c r="D23" s="28"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="30"/>
+      <c r="B24" s="28" t="s">
+        <v>311</v>
+      </c>
+      <c r="C24" s="57"/>
+      <c r="D24" s="28"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="30"/>
+      <c r="B25" s="28" t="s">
+        <v>318</v>
+      </c>
+      <c r="C25" s="57"/>
+      <c r="D25" s="28"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="30"/>
+      <c r="B26" s="28" t="s">
+        <v>314</v>
+      </c>
+      <c r="C26" s="57"/>
+      <c r="D26" s="28"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="30"/>
+      <c r="B27" s="28" t="s">
+        <v>315</v>
+      </c>
+      <c r="C27" s="57"/>
+      <c r="D27" s="28"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="30"/>
+      <c r="B28" s="28" t="s">
+        <v>316</v>
+      </c>
+      <c r="C28" s="57"/>
+      <c r="D28" s="28"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="30"/>
+      <c r="B29" s="28" t="s">
+        <v>317</v>
+      </c>
+      <c r="C29" s="57"/>
+      <c r="D29" s="28"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="30"/>
+      <c r="C30" s="57"/>
+      <c r="D30" s="28"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="30" t="s">
+        <v>289</v>
+      </c>
+      <c r="B31" s="56"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="30"/>
+      <c r="B32" s="56" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="30" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="B34" s="28" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="30" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B36" s="28" t="s">
+        <v>103</v>
+      </c>
+      <c r="C36" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D36" s="28" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B37" s="28" t="s">
+        <v>104</v>
+      </c>
+      <c r="C37" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D37" s="28" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B38" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="C38" s="57" t="s">
+        <v>204</v>
+      </c>
+      <c r="D38" s="28" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="30" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="48" t="s">
+        <v>103</v>
+      </c>
+      <c r="B40" s="49" t="s">
+        <v>104</v>
+      </c>
+      <c r="C40" s="49" t="s">
+        <v>105</v>
+      </c>
+      <c r="D40" s="55" t="s">
+        <v>176</v>
+      </c>
+      <c r="E40" s="49" t="s">
+        <v>130</v>
+      </c>
+      <c r="F40" s="50" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+      <c r="A41" s="51" t="s">
+        <v>107</v>
+      </c>
+      <c r="B41" s="36" t="s">
+        <v>109</v>
+      </c>
+      <c r="C41" s="36">
+        <v>1</v>
+      </c>
+      <c r="D41" s="37" t="s">
+        <v>177</v>
+      </c>
+      <c r="E41" s="37" t="s">
+        <v>154</v>
+      </c>
+      <c r="F41" s="52" t="s">
+        <v>110</v>
+      </c>
+      <c r="G41" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+      <c r="A42" s="42" t="s">
+        <v>111</v>
+      </c>
+      <c r="B42" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C42" s="32">
+        <v>0</v>
+      </c>
+      <c r="D42" s="33" t="s">
+        <v>178</v>
+      </c>
+      <c r="E42" s="33" t="s">
+        <v>155</v>
+      </c>
+      <c r="F42" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="G42" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A43" s="42" t="s">
+        <v>112</v>
+      </c>
+      <c r="B43" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C43" s="32">
+        <v>30</v>
+      </c>
+      <c r="D43" s="33" t="s">
+        <v>179</v>
+      </c>
+      <c r="E43" s="33" t="s">
+        <v>156</v>
+      </c>
+      <c r="F43" s="43" t="s">
+        <v>114</v>
+      </c>
+      <c r="G43" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+      <c r="A44" s="42" t="s">
+        <v>113</v>
+      </c>
+      <c r="B44" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C44" s="32">
+        <v>30</v>
+      </c>
+      <c r="D44" s="33" t="s">
+        <v>180</v>
+      </c>
+      <c r="E44" s="33" t="s">
+        <v>158</v>
+      </c>
+      <c r="F44" s="43" t="s">
+        <v>157</v>
+      </c>
+      <c r="G44" s="28" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A45" s="42" t="s">
+        <v>116</v>
+      </c>
+      <c r="B45" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C45" s="32">
+        <v>30</v>
+      </c>
+      <c r="D45" s="33" t="s">
+        <v>181</v>
+      </c>
+      <c r="E45" s="33" t="s">
+        <v>159</v>
+      </c>
+      <c r="F45" s="43" t="s">
+        <v>114</v>
+      </c>
+      <c r="G45" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A46" s="42" t="s">
+        <v>117</v>
+      </c>
+      <c r="B46" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C46" s="32">
+        <v>30</v>
+      </c>
+      <c r="D46" s="33" t="s">
+        <v>182</v>
+      </c>
+      <c r="E46" s="33" t="s">
+        <v>160</v>
+      </c>
+      <c r="F46" s="43" t="s">
+        <v>161</v>
+      </c>
+      <c r="G46" s="28" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="89.25" x14ac:dyDescent="0.25">
+      <c r="A47" s="42" t="s">
+        <v>136</v>
+      </c>
+      <c r="B47" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C47" s="32">
+        <v>1</v>
+      </c>
+      <c r="D47" s="33" t="s">
+        <v>184</v>
+      </c>
+      <c r="E47" s="33" t="s">
+        <v>162</v>
+      </c>
+      <c r="F47" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="G47" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A48" s="42" t="s">
+        <v>132</v>
+      </c>
+      <c r="B48" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C48" s="32">
+        <v>72</v>
+      </c>
+      <c r="D48" s="33" t="s">
+        <v>183</v>
+      </c>
+      <c r="E48" s="33" t="s">
+        <v>146</v>
+      </c>
+      <c r="F48" s="43" t="s">
+        <v>134</v>
+      </c>
+      <c r="G48" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="89.25" x14ac:dyDescent="0.25">
+      <c r="A49" s="42" t="s">
+        <v>137</v>
+      </c>
+      <c r="B49" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C49" s="32">
+        <v>0</v>
+      </c>
+      <c r="D49" s="33" t="s">
+        <v>185</v>
+      </c>
+      <c r="E49" s="33" t="s">
+        <v>163</v>
+      </c>
+      <c r="F49" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="G49" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="53" t="s">
+        <v>133</v>
+      </c>
+      <c r="B50" s="34" t="s">
+        <v>109</v>
+      </c>
+      <c r="C50" s="34">
+        <v>69</v>
+      </c>
+      <c r="D50" s="35" t="s">
+        <v>186</v>
+      </c>
+      <c r="E50" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="F50" s="54" t="s">
+        <v>135</v>
+      </c>
+      <c r="G50" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="191.25" x14ac:dyDescent="0.25">
+      <c r="A51" s="38" t="s">
+        <v>118</v>
+      </c>
+      <c r="B51" s="39" t="s">
+        <v>109</v>
+      </c>
+      <c r="C51" s="39">
+        <v>2</v>
+      </c>
+      <c r="D51" s="40" t="s">
+        <v>187</v>
+      </c>
+      <c r="E51" s="40" t="s">
+        <v>164</v>
+      </c>
+      <c r="F51" s="41" t="s">
+        <v>166</v>
+      </c>
+      <c r="G51" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="42" t="s">
+        <v>119</v>
+      </c>
+      <c r="B52" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C52" s="32">
+        <v>54</v>
+      </c>
+      <c r="D52" s="33" t="s">
+        <v>189</v>
+      </c>
+      <c r="E52" s="33" t="s">
+        <v>148</v>
+      </c>
+      <c r="F52" s="43" t="s">
+        <v>120</v>
+      </c>
+      <c r="G52" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="178.5" x14ac:dyDescent="0.25">
+      <c r="A53" s="42" t="s">
+        <v>121</v>
+      </c>
+      <c r="B53" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C53" s="32">
+        <v>1</v>
+      </c>
+      <c r="D53" s="33" t="s">
+        <v>188</v>
+      </c>
+      <c r="E53" s="33" t="s">
+        <v>165</v>
+      </c>
+      <c r="F53" s="41" t="s">
+        <v>431</v>
+      </c>
+      <c r="G53" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="53" t="s">
+        <v>122</v>
+      </c>
+      <c r="B54" s="34" t="s">
+        <v>109</v>
+      </c>
+      <c r="C54" s="34">
+        <v>44</v>
+      </c>
+      <c r="D54" s="35" t="s">
+        <v>189</v>
+      </c>
+      <c r="E54" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="F54" s="54" t="s">
+        <v>123</v>
+      </c>
+      <c r="G54" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+      <c r="A55" s="38" t="s">
+        <v>127</v>
+      </c>
+      <c r="B55" s="39" t="s">
+        <v>109</v>
+      </c>
+      <c r="C55" s="39">
+        <v>1</v>
+      </c>
+      <c r="D55" s="40" t="s">
+        <v>191</v>
+      </c>
+      <c r="E55" s="40" t="s">
+        <v>167</v>
+      </c>
+      <c r="F55" s="41" t="s">
+        <v>110</v>
+      </c>
+      <c r="G55" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A56" s="42" t="s">
+        <v>125</v>
+      </c>
+      <c r="B56" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C56" s="32">
+        <v>42</v>
+      </c>
+      <c r="D56" s="33" t="s">
+        <v>189</v>
+      </c>
+      <c r="E56" s="33" t="s">
+        <v>150</v>
+      </c>
+      <c r="F56" s="43" t="s">
+        <v>128</v>
+      </c>
+      <c r="G56" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+      <c r="A57" s="42" t="s">
+        <v>126</v>
+      </c>
+      <c r="B57" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C57" s="32">
+        <v>0</v>
+      </c>
+      <c r="D57" s="33" t="s">
+        <v>190</v>
+      </c>
+      <c r="E57" s="33" t="s">
+        <v>168</v>
+      </c>
+      <c r="F57" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="G57" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="44" t="s">
+        <v>124</v>
+      </c>
+      <c r="B58" s="45" t="s">
+        <v>109</v>
+      </c>
+      <c r="C58" s="45">
+        <v>38</v>
+      </c>
+      <c r="D58" s="46" t="s">
+        <v>189</v>
+      </c>
+      <c r="E58" s="46" t="s">
+        <v>151</v>
+      </c>
+      <c r="F58" s="47" t="s">
+        <v>129</v>
+      </c>
+      <c r="G58" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="153" x14ac:dyDescent="0.25">
+      <c r="A59" s="51" t="s">
+        <v>138</v>
+      </c>
+      <c r="B59" s="36" t="s">
+        <v>109</v>
+      </c>
+      <c r="C59" s="36">
+        <v>1</v>
+      </c>
+      <c r="D59" s="37" t="s">
+        <v>192</v>
+      </c>
+      <c r="E59" s="37" t="s">
+        <v>169</v>
+      </c>
+      <c r="F59" s="52" t="s">
+        <v>110</v>
+      </c>
+      <c r="G59" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+      <c r="A60" s="42" t="s">
+        <v>143</v>
+      </c>
+      <c r="B60" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C60" s="32">
+        <v>0</v>
+      </c>
+      <c r="D60" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="E60" s="33" t="s">
+        <v>152</v>
+      </c>
+      <c r="F60" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="G60" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="90" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="44" t="s">
+        <v>142</v>
+      </c>
+      <c r="B61" s="45" t="s">
+        <v>109</v>
+      </c>
+      <c r="C61" s="45">
+        <v>50</v>
+      </c>
+      <c r="D61" s="46" t="s">
+        <v>194</v>
+      </c>
+      <c r="E61" s="46" t="s">
+        <v>170</v>
+      </c>
+      <c r="F61" s="47" t="s">
+        <v>144</v>
+      </c>
+      <c r="G61" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="216.75" x14ac:dyDescent="0.25">
+      <c r="A62" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="B62" s="39" t="s">
+        <v>109</v>
+      </c>
+      <c r="C62" s="39">
+        <v>1</v>
+      </c>
+      <c r="D62" s="40" t="s">
+        <v>195</v>
+      </c>
+      <c r="E62" s="40" t="s">
+        <v>175</v>
+      </c>
+      <c r="F62" s="41" t="s">
+        <v>110</v>
+      </c>
+      <c r="G62" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+      <c r="A63" s="42" t="s">
+        <v>140</v>
+      </c>
+      <c r="B63" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="C63" s="32">
+        <v>0</v>
+      </c>
+      <c r="D63" s="33" t="s">
+        <v>196</v>
+      </c>
+      <c r="E63" s="33" t="s">
+        <v>153</v>
+      </c>
+      <c r="F63" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="G63" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" ht="90" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="53" t="s">
+        <v>141</v>
+      </c>
+      <c r="B64" s="34" t="s">
+        <v>109</v>
+      </c>
+      <c r="C64" s="34">
+        <v>60</v>
+      </c>
+      <c r="D64" s="35" t="s">
+        <v>197</v>
+      </c>
+      <c r="E64" s="35" t="s">
+        <v>171</v>
+      </c>
+      <c r="F64" s="54" t="s">
+        <v>145</v>
+      </c>
+      <c r="G64" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A65" s="38" t="s">
         <v>172</v>
       </c>
@@ -4472,8 +8627,11 @@
       <c r="F65" s="41" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" ht="102.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G65" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="102.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="44" t="s">
         <v>173</v>
       </c>
@@ -4492,23 +8650,26 @@
       <c r="F66" s="47" t="s">
         <v>416</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G66" s="28" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="30" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B69" s="28" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="30" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="30" t="s">
         <v>102</v>
       </c>
@@ -4516,12 +8677,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="30" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B73" s="28" t="s">
         <v>205</v>
       </c>
@@ -4532,7 +8693,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B74" s="28" t="s">
         <v>206</v>
       </c>
@@ -4543,7 +8704,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B75" s="28" t="s">
         <v>207</v>
       </c>
@@ -4554,7 +8715,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B76" s="28" t="s">
         <v>208</v>
       </c>
@@ -4565,7 +8726,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B77" s="28" t="s">
         <v>209</v>
       </c>
@@ -4576,7 +8737,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B78" s="28" t="s">
         <v>210</v>
       </c>
@@ -4587,7 +8748,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B79" s="28" t="s">
         <v>211</v>
       </c>
@@ -4598,7 +8759,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="30" t="s">
         <v>217</v>
       </c>
@@ -5602,10 +9763,10 @@
       </c>
     </row>
     <row r="217" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D217" s="72" t="s">
+      <c r="D217" s="73" t="s">
         <v>419</v>
       </c>
-      <c r="E217" s="72"/>
+      <c r="E217" s="73"/>
     </row>
     <row r="218" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C218" s="58" t="s">
@@ -5615,10 +9776,10 @@
       <c r="E218" s="63"/>
     </row>
     <row r="219" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="D219" s="72" t="s">
+      <c r="D219" s="73" t="s">
         <v>420</v>
       </c>
-      <c r="E219" s="72"/>
+      <c r="E219" s="73"/>
     </row>
     <row r="220" spans="3:5" x14ac:dyDescent="0.25">
       <c r="C220" s="28" t="s">

</xml_diff>